<commit_message>
Update answer key; fix typo in inter-rater rating template
</commit_message>
<xml_diff>
--- a/02_detection_reliability/DEPOSIT_inter_rater_ratings_template.xlsx
+++ b/02_detection_reliability/DEPOSIT_inter_rater_ratings_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiwon/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62DFFDE-4A03-4247-A815-C43DCBD94D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A506F40-1A82-AA42-A0E3-B9087D3A6E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -729,15 +729,6 @@
     <t>· In each of the KBI / KRA / GeNA cells, enter one of the following (click the cell for a drop-down).</t>
   </si>
   <si>
-    <t xml:space="preserve">     예 (Yes)          = No problem (the file passes this checkpoint)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     아니오 (No)        = Defect found (the file does not pass this checkpoint)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     해당없음 (N/A)    = Not applicable to that data type (e.g., a genomics-only item applied to an imaging file)</t>
-  </si>
-  <si>
     <t>· Items are presented in both English and Korean. In the 'Basis for judgment' cell, please note the evidence for your decision, such as the row or field where you found the problem (optional).</t>
   </si>
   <si>
@@ -762,16 +753,25 @@
     <t>Date of rating:</t>
   </si>
   <si>
-    <t xml:space="preserve"> KBI (Yes/No/No applicable)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> KRA (Yes/No/No applicable)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> GeNA (Yes/No/No applicable)</t>
-  </si>
-  <si>
     <t>Reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KBI (Pass/Fail/No applicable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KRA (Pass/Fail/No applicable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> GeNA (Pass/Fail/No applicable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     예 (Pass)          = No problem (the file passes this checkpoint)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     아니오 (Fail)        = Defect found (the file does not pass this checkpoint)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     해당없음 (No applicable)    = Not applicable to that data type (e.g., a genomics-only item applied to an imaging file)</t>
   </si>
 </sst>
 </file>
@@ -1490,22 +1490,22 @@
     </row>
     <row r="18" spans="2:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="21" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B19" s="21" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B20" s="21" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="32" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.2">
@@ -1513,22 +1513,22 @@
     </row>
     <row r="23" spans="2:2" ht="17" x14ac:dyDescent="0.2">
       <c r="B23" s="20" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="2:2" ht="32" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="2:2" ht="32" x14ac:dyDescent="0.2">
       <c r="B26" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.2">
@@ -1536,17 +1536,17 @@
     </row>
     <row r="28" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B28" s="21" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B29" s="21" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="30" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B30" s="21" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1590,16 +1590,16 @@
         <v>5</v>
       </c>
       <c r="G1" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="H1" s="13" t="s">
-        <v>237</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>238</v>
-      </c>
       <c r="J1" s="14" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>